<commit_message>
EPBDS-16292 Fix wrong and lost parameter-field inputs in trace step details
</commit_message>
<xml_diff>
--- a/STUDIO/org.openl.rules.webstudio/test/rules/trace-debug/fieldAccessProject.xlsx
+++ b/STUDIO/org.openl.rules.webstudio/test/rules/trace-debug/fieldAccessProject.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,11 +529,43 @@
         <v>5</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Spreadsheet Integer TwoPolicies ( Policy prior, Policy current )</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Pick</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>= CountCensus ( current.census )</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A1:B1"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A1:B1"/>
     <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>